<commit_message>
mise à jour cours Kurbenete et réseau
</commit_message>
<xml_diff>
--- a/RESEAU/RESEAU_Liste _commande.xlsx
+++ b/RESEAU/RESEAU_Liste _commande.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a5f61b3e4cd8107/Documents/M2i_AdministrateurCLOUD/Cours_les_reseaux/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a5f61b3e4cd8107/Inès_perso/M2i_administraeur_CLOUD.0.0/Cours_Python_M2i/RESEAU/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="100" documentId="8_{6A324A7E-F49D-4A31-95DF-2C9C17B80965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{423D5C3F-9DA3-4EA6-B293-16C2B731F883}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="8_{6A324A7E-F49D-4A31-95DF-2C9C17B80965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71833836-3410-4D3B-9752-B841DFF714D4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{53579A57-D536-4490-91DF-98FD1ABCE521}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Action</t>
   </si>
@@ -307,6 +307,12 @@
   <si>
     <t>qui écoute en TCP sur ma machine ? (vu en CL-LINUX)</t>
   </si>
+  <si>
+    <t>HTTP/1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     GET /produits HTTP/1.1  </t>
+  </si>
 </sst>
 </file>
 
@@ -640,6 +646,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -651,15 +666,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -676,10 +682,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1041,7 +1043,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="24" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -1052,7 +1054,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="21"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1081,7 +1083,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="25" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -1092,7 +1094,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="23"/>
+      <c r="A9" s="26"/>
       <c r="B9" s="2" t="s">
         <v>22</v>
       </c>
@@ -1101,7 +1103,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="24"/>
+      <c r="A10" s="27"/>
       <c r="B10" s="14" t="s">
         <v>24</v>
       </c>
@@ -1121,7 +1123,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="25" t="s">
         <v>29</v>
       </c>
       <c r="B12" s="11" t="s">
@@ -1132,7 +1134,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
+      <c r="A13" s="26"/>
       <c r="B13" s="19" t="s">
         <v>32</v>
       </c>
@@ -1141,7 +1143,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="23"/>
+      <c r="A14" s="26"/>
       <c r="B14" s="2" t="s">
         <v>34</v>
       </c>
@@ -1150,7 +1152,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="23"/>
+      <c r="A15" s="26"/>
       <c r="B15" s="2" t="s">
         <v>36</v>
       </c>
@@ -1159,7 +1161,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="23"/>
+      <c r="A16" s="26"/>
       <c r="B16" s="2" t="s">
         <v>38</v>
       </c>
@@ -1168,7 +1170,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="23"/>
+      <c r="A17" s="26"/>
       <c r="B17" s="2" t="s">
         <v>40</v>
       </c>
@@ -1177,7 +1179,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="127.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="24"/>
+      <c r="A18" s="27"/>
       <c r="B18" s="14" t="s">
         <v>42</v>
       </c>
@@ -1186,18 +1188,18 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="23" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="21" t="s">
         <v>47</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -1208,8 +1210,12 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="8"/>
-      <c r="B21" s="2"/>
+      <c r="A21" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="C21" s="2"/>
     </row>
   </sheetData>

</xml_diff>